<commit_message>
Update: sector filtering, structure filter, framework matrix
</commit_message>
<xml_diff>
--- a/data/MEL_Indicator_Reference.xlsx
+++ b/data/MEL_Indicator_Reference.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MEL_Indicators" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Species_by_Sector" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure_by_Sector" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3182,6 +3183,312 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Aquaculture Type</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Farm Structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Longline (surface)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Longline (subsurface)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Raft / floating</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Off-bottom (monoline / pegs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Bottom culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Land-based tank or pond</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>IMTA infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Seaweed</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Floating cage / tray</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Bouchot / pole culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Intertidal rack-and-bag</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Trestle / trays (intertidal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>On-bottom cages</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Suspended lantern net</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Suspended longline (mussel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Pearl net / spat collector</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Floating bag (oyster)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Off-bottom suspended oyster (BC-style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Intertidal net-over-substrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Raft / hanging rope</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Bottom culture (clam seeded substrate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Mollusk</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Reef / on-bottom structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Not gear-specific</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>